<commit_message>
Translator workbook: add 'Date formats' sheet (samples per language, 12-hour rule)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Cvent Code Files/Cvent Widgets/Widget Playbook & Boilerplate/agenda-widget-translations.xlsx
+++ b/Cvent Code Files/Cvent Widgets/Widget Playbook & Boilerplate/agenda-widget-translations.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Read me" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Strings" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Date formats" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -579,7 +580,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>6. The 'Locale code' row is not a translation — it tells the browser how to format DATES (month and weekday names). Times are always shown on a 12-hour clock in every language, by decision.</t>
+          <t>6. The 'Locale code' row on 'Strings' tells the browser how to format DATES; the 'Date formats' sheet shows every date pattern with sample output per language so translators can confirm the locale and expected wording. Times are always 12-hour, by decision.</t>
         </is>
       </c>
     </row>
@@ -1572,4 +1573,389 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Where it appears</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Pattern (what the browser is asked for)</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>English — locale en-US</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Spanish — locale es</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Portuguese — locale pt-BR</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Japanese — locale ja-JP?</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Chinese (Mandarin) — locale zh-CN?</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>Korean — locale ko-KR?</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>French — locale fr-FR?</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>German — locale de-DE?</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>dayHeader</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>Day header above each day's sessions</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>weekday long, day, month long — first letter capitalised</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>Monday, June 16</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>Lunes, 16 de junio</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>Segunda-feira, 16 de junho</t>
+        </is>
+      </c>
+      <c r="G2" s="8" t="inlineStr"/>
+      <c r="H2" s="8" t="inlineStr"/>
+      <c r="I2" s="8" t="inlineStr"/>
+      <c r="J2" s="8" t="inlineStr"/>
+      <c r="K2" s="8" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>dateTab</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Date navigation tab (Editorial header): weekday / day / month stacked</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>weekday short · day · month short, no trailing dots</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>Mon · 16 · Jun</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>lun · 16 · jun</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>seg · 16 · jun</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr"/>
+      <c r="H3" s="8" t="inlineStr"/>
+      <c r="I3" s="8" t="inlineStr"/>
+      <c r="J3" s="8" t="inlineStr"/>
+      <c r="K3" s="8" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dateTabClassic</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Date navigation link (Classic header)</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>weekday long, day, month long</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Monday, June 16</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>Lunes, 16 de junio</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>Segunda-feira, 16 de junho</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="inlineStr"/>
+      <c r="H4" s="8" t="inlineStr"/>
+      <c r="I4" s="8" t="inlineStr"/>
+      <c r="J4" s="8" t="inlineStr"/>
+      <c r="K4" s="8" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>eyebrowRange</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Editorial header eyebrow when the planner leaves it blank: first day – last day</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>month short, day (+ year when it differs / on the last day)</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Jun 16, 2025 – Dec 31, 2026</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>16 jun 2025 – 31 dic 2026</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>16 de jun. de 2025 – 31 de dez. de 2026</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="inlineStr"/>
+      <c r="H5" s="8" t="inlineStr"/>
+      <c r="I5" s="8" t="inlineStr"/>
+      <c r="J5" s="8" t="inlineStr"/>
+      <c r="K5" s="8" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>sessionModalDateLine</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Line under the title in the session modal</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>weekday short, month short, day — then the 12-hour time range</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Mon, Jun 16, 10:00 AM – 11:00 AM</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>Lun, 16 jun, 10:00 AM – 11:00 AM</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>Seg., 16 de jun., 10:00 AM – 11:00 AM</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="inlineStr"/>
+      <c r="H6" s="8" t="inlineStr"/>
+      <c r="I6" s="8" t="inlineStr"/>
+      <c r="J6" s="8" t="inlineStr"/>
+      <c r="K6" s="8" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>speakerModalSessionDate</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Each session in the speaker modal's Sessions list</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>month short, day, year — then the 12-hour time range</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Jun 16, 2025, 9:45 AM – 10:30 AM GMT+2</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>16 jun 2025, 9:45 AM – 10:30 AM GMT+2</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>16 de jun. de 2025, 9:45 AM – 10:30 AM GMT+2</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr"/>
+      <c r="H7" s="8" t="inlineStr"/>
+      <c r="I7" s="8" t="inlineStr"/>
+      <c r="J7" s="8" t="inlineStr"/>
+      <c r="K7" s="8" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>times</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Every time on cards, tiles, the time rail, and both modals</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>ALWAYS 12-hour with AM/PM, in every language (by decision)</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>9:45 AM–10:30 AM</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>9:45 AM–10:30 AM</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>9:45 AM–10:30 AM</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="inlineStr"/>
+      <c r="H8" s="8" t="inlineStr"/>
+      <c r="I8" s="8" t="inlineStr"/>
+      <c r="J8" s="8" t="inlineStr"/>
+      <c r="K8" s="8" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>How to use this sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>These are NOT typed translations. The browser builds each date from the locale code in the column header, so the grey cells show what English, Spanish and Portuguese attendees see today.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>For each new language: (1) confirm or correct the locale code in the header (the '?' marks a suggested default — e.g. zh-TW instead of zh-CN if the audience is Taiwan); (2) in the yellow cells, write the date as it SHOULD read for that pattern, so we can check the browser's output against a native expectation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Times are always 12-hour with AM/PM in every language. That is a deliberate decision; do not propose 24-hour variants here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Time zone abbreviations (GMT+2 etc.) are supplied by the browser and are not translated.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A11:F11"/>
+    <mergeCell ref="A10:F10"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A12:F12"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Opt-in session filters: type / location / category / tags
A chip bar under the date nav (showFilters, default off, in New Features).
Each facet is a checkbox menu; a facet appears only when the agenda has two
or more values for it. Type uses the planner's plenary / focus labels and
hides breaks when chosen. AND across facets, OR within. Nav tabs, eyebrow
and 'appears in' lists use all sessions; only the rendered day sections are
filtered; an empty state with 'Clear filters' shows when nothing matches.
Re-renders now reuse a session cache keyed by sort + page size, so filtering
(and config changes) never refetch. Six new UI strings added to the en/es/pt
tables and the translator workbook.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Cvent Code Files/Cvent Widgets/Widget Playbook & Boilerplate/agenda-widget-translations.xlsx
+++ b/Cvent Code Files/Cvent Widgets/Widget Playbook & Boilerplate/agenda-widget-translations.xlsx
@@ -629,7 +629,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K28"/>
+  <dimension ref="A1:K34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1482,83 +1482,306 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
+          <t>filterType</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>Filter chip label in the session filter bar (values are the plenary / focus labels)</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr"/>
+      <c r="H23" s="8" t="inlineStr"/>
+      <c r="I23" s="8" t="inlineStr"/>
+      <c r="J23" s="8" t="inlineStr"/>
+      <c r="K23" s="8" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>filterLocation</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>Filter chip label</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>Ubicación</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr"/>
+      <c r="H24" s="8" t="inlineStr"/>
+      <c r="I24" s="8" t="inlineStr"/>
+      <c r="J24" s="8" t="inlineStr"/>
+      <c r="K24" s="8" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>filterCategory</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>Filter chip label</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>Categoría</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>Categoria</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr"/>
+      <c r="H25" s="8" t="inlineStr"/>
+      <c r="I25" s="8" t="inlineStr"/>
+      <c r="J25" s="8" t="inlineStr"/>
+      <c r="K25" s="8" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>filterTags</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>Filter chip label</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>Tags</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>Etiquetas</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>Tags</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr"/>
+      <c r="H26" s="8" t="inlineStr"/>
+      <c r="I26" s="8" t="inlineStr"/>
+      <c r="J26" s="8" t="inlineStr"/>
+      <c r="K26" s="8" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>clearFilters</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>Link that resets all session filters</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>phrase</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>Clear filters</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>Borrar filtros</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>Limpar filtros</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr"/>
+      <c r="H27" s="8" t="inlineStr"/>
+      <c r="I27" s="8" t="inlineStr"/>
+      <c r="J27" s="8" t="inlineStr"/>
+      <c r="K27" s="8" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>noMatches</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>Message when the chosen filters leave no sessions to show</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>sentence</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>No sessions match these filters.</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>Ninguna sesión coincide con estos filtros.</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>Nenhuma sessão corresponde a estes filtros.</t>
+        </is>
+      </c>
+      <c r="G28" s="8" t="inlineStr"/>
+      <c r="H28" s="8" t="inlineStr"/>
+      <c r="I28" s="8" t="inlineStr"/>
+      <c r="J28" s="8" t="inlineStr"/>
+      <c r="K28" s="8" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
           <t>localeCode</t>
         </is>
       </c>
-      <c r="B23" s="6" t="inlineStr">
+      <c r="B29" s="6" t="inlineStr">
         <is>
           <t>NOT a translation: BCP-47 locale the browser uses to format dates (month and weekday names). Times stay 12-hour.</t>
         </is>
       </c>
-      <c r="C23" s="6" t="inlineStr">
+      <c r="C29" s="6" t="inlineStr">
         <is>
           <t>locale code</t>
         </is>
       </c>
-      <c r="D23" s="7" t="inlineStr">
+      <c r="D29" s="7" t="inlineStr">
         <is>
           <t>en-US</t>
         </is>
       </c>
-      <c r="E23" s="7" t="inlineStr">
+      <c r="E29" s="7" t="inlineStr">
         <is>
           <t>es</t>
         </is>
       </c>
-      <c r="F23" s="7" t="inlineStr">
+      <c r="F29" s="7" t="inlineStr">
         <is>
           <t>pt-BR</t>
         </is>
       </c>
-      <c r="G23" s="8" t="inlineStr">
+      <c r="G29" s="8" t="inlineStr">
         <is>
           <t>ja-JP</t>
         </is>
       </c>
-      <c r="H23" s="8" t="inlineStr">
+      <c r="H29" s="8" t="inlineStr">
         <is>
           <t>zh-CN</t>
         </is>
       </c>
-      <c r="I23" s="8" t="inlineStr">
+      <c r="I29" s="8" t="inlineStr">
         <is>
           <t>ko-KR</t>
         </is>
       </c>
-      <c r="J23" s="8" t="inlineStr">
+      <c r="J29" s="8" t="inlineStr">
         <is>
           <t>fr-FR</t>
         </is>
       </c>
-      <c r="K23" s="8" t="inlineStr">
+      <c r="K29" s="8" t="inlineStr">
         <is>
           <t>de-DE</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+    <row r="30"/>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>Legend</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="9" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="9" t="inlineStr">
         <is>
           <t>Shipped in code today (reference — do not edit here)</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="10" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="10" t="inlineStr">
         <is>
           <t>To be filled in by translators (blank = English is used)</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="11" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="11" t="inlineStr">
         <is>
           <t>The five locale codes on the last row are suggested defaults; confirm the regional variant (e.g. zh-TW vs zh-CN, fr-CA vs fr-FR) if the audience needs it.</t>
         </is>

</xml_diff>